<commit_message>
Update sample test data in input.xlsx
Shared sample table list, kept up to date for anyone trying the app.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amedeloitte-my.sharepoint.com/personal/ritwichatterjee_deloitte_com/Documents/Desktop/SAP Assessment Automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{E90854E9-3B04-4FBA-90F0-76CB91019839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E52224C2-5E0A-4A1E-96A4-E918F33012B6}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{E90854E9-3B04-4FBA-90F0-76CB91019839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E697455C-F3A8-4C99-82F6-A470C5CABA6A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{2B194D51-A276-444F-BEB8-1EF57CE1E639}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="92">
   <si>
     <t>BKPF</t>
   </si>
@@ -105,6 +105,216 @@
   </si>
   <si>
     <t>DESCRIPTION</t>
+  </si>
+  <si>
+    <t>COSP</t>
+  </si>
+  <si>
+    <t>COSS</t>
+  </si>
+  <si>
+    <t>GLPCP</t>
+  </si>
+  <si>
+    <t>VBKD</t>
+  </si>
+  <si>
+    <t>VBRP</t>
+  </si>
+  <si>
+    <t>GLPCA</t>
+  </si>
+  <si>
+    <t>CDPOS</t>
+  </si>
+  <si>
+    <t>COBK</t>
+  </si>
+  <si>
+    <t>LIPS</t>
+  </si>
+  <si>
+    <t>RSPMDATAPID</t>
+  </si>
+  <si>
+    <t>SRRELROLES</t>
+  </si>
+  <si>
+    <t>ARFCSDATA</t>
+  </si>
+  <si>
+    <t>VRPMA</t>
+  </si>
+  <si>
+    <t>VAPMA</t>
+  </si>
+  <si>
+    <t>SWNCMONI</t>
+  </si>
+  <si>
+    <t>DFKKZR</t>
+  </si>
+  <si>
+    <t>ODQDATA</t>
+  </si>
+  <si>
+    <t>BALDAT</t>
+  </si>
+  <si>
+    <t>SWWLOGHIST</t>
+  </si>
+  <si>
+    <t>EDIDS</t>
+  </si>
+  <si>
+    <t>UJ0_STAT_DTL</t>
+  </si>
+  <si>
+    <t>ETXDCH</t>
+  </si>
+  <si>
+    <t>ETXDCI</t>
+  </si>
+  <si>
+    <t>ETXDCJ</t>
+  </si>
+  <si>
+    <t>SWFREVTLOG</t>
+  </si>
+  <si>
+    <t>KONV</t>
+  </si>
+  <si>
+    <t>RSDDSTATEVDATA</t>
+  </si>
+  <si>
+    <t>RSBATCHDATA</t>
+  </si>
+  <si>
+    <t>RSMONMESS</t>
+  </si>
+  <si>
+    <t>DBTABLOG</t>
+  </si>
+  <si>
+    <t>CKMI1</t>
+  </si>
+  <si>
+    <t>EDID4</t>
+  </si>
+  <si>
+    <t>BALHDR</t>
+  </si>
+  <si>
+    <t>EBAN</t>
+  </si>
+  <si>
+    <t>BSAD</t>
+  </si>
+  <si>
+    <t>BSAS</t>
+  </si>
+  <si>
+    <t>BSIS</t>
+  </si>
+  <si>
+    <t>Generated Table for View</t>
+  </si>
+  <si>
+    <t>EC-PCA: Plan Line Items</t>
+  </si>
+  <si>
+    <t>Sales Document: Business Data</t>
+  </si>
+  <si>
+    <t>Billing Document: Item Data</t>
+  </si>
+  <si>
+    <t>EC-PCA: Actual Line Items</t>
+  </si>
+  <si>
+    <t>Change document items</t>
+  </si>
+  <si>
+    <t>CO Object: Document Header</t>
+  </si>
+  <si>
+    <t>SD document: Delivery: Item data</t>
+  </si>
+  <si>
+    <t>RSPM Data Package</t>
+  </si>
+  <si>
+    <t>Object Relationship Service: Roles</t>
+  </si>
+  <si>
+    <t>ARFC Call Data (Callers)</t>
+  </si>
+  <si>
+    <t>SD Index: Billing Items per Material</t>
+  </si>
+  <si>
+    <t>Sales Index: Order Items by Material</t>
+  </si>
+  <si>
+    <t>SAP Workload NW Collector: Data Clusters</t>
+  </si>
+  <si>
+    <t>Payment form</t>
+  </si>
+  <si>
+    <t>Operational Delta Queue: Data Store for Delta</t>
+  </si>
+  <si>
+    <t>Application Log: Log data</t>
+  </si>
+  <si>
+    <t>Workflow Runtime: History of a Work Item</t>
+  </si>
+  <si>
+    <t>Status Record (IDoc)</t>
+  </si>
+  <si>
+    <t>BPC: Statistics Detailed Info</t>
+  </si>
+  <si>
+    <t>External tax document: header info</t>
+  </si>
+  <si>
+    <t>External tax document: line item info</t>
+  </si>
+  <si>
+    <t>Ext. tax document: tax rates and amounts by Jurisdict. level</t>
+  </si>
+  <si>
+    <t>Event Log</t>
+  </si>
+  <si>
+    <t>Conditions (Obsolete - replaced by PRCD_ELEMENTS)</t>
+  </si>
+  <si>
+    <t>BW Statistics (OLAP), Key Figures for the Events</t>
+  </si>
+  <si>
+    <t>Copy of INDX for Batch and Enqueue Runtime Data</t>
+  </si>
+  <si>
+    <t>Messages for the monitor</t>
+  </si>
+  <si>
+    <t>Log Records of Table Changes</t>
+  </si>
+  <si>
+    <t>Index for Accounting Documents for Material</t>
+  </si>
+  <si>
+    <t>IDoc Data Records from 4.0 onwards</t>
+  </si>
+  <si>
+    <t>Application log: log header</t>
+  </si>
+  <si>
+    <t>Purchase Requisition</t>
   </si>
 </sst>
 </file>
@@ -153,9 +363,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -492,10 +708,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{797D741F-F08F-46C6-8A1B-2BEDC41FD56F}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.90625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -508,83 +724,379 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B4" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B8" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B11" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B13" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B33" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A46" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A47" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B47" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A48" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B48" s="3" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>